<commit_message>
Initial commit for new repository
</commit_message>
<xml_diff>
--- a/all_CLients.xlsx
+++ b/all_CLients.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Client Name</t>
   </si>
@@ -25,40 +25,94 @@
     <t>CLient NationalID</t>
   </si>
   <si>
-    <t>mahmoud</t>
-  </si>
-  <si>
-    <t>mahmoud@gmail.com</t>
-  </si>
-  <si>
-    <t>2123213124</t>
-  </si>
-  <si>
-    <t>ahmed</t>
-  </si>
-  <si>
-    <t>ahmed@gmail.com</t>
-  </si>
-  <si>
-    <t>21232674676</t>
-  </si>
-  <si>
-    <t>jack</t>
-  </si>
-  <si>
-    <t>jack22@gmail.com</t>
-  </si>
-  <si>
-    <t>123142423</t>
-  </si>
-  <si>
-    <t>john33</t>
-  </si>
-  <si>
-    <t>john33@gmail.com</t>
-  </si>
-  <si>
-    <t>4534636346</t>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>alice@example.com</t>
+  </si>
+  <si>
+    <t>123456789</t>
+  </si>
+  <si>
+    <t>Bob</t>
+  </si>
+  <si>
+    <t>bob@example.com</t>
+  </si>
+  <si>
+    <t>987654321</t>
+  </si>
+  <si>
+    <t>Charlie</t>
+  </si>
+  <si>
+    <t>charlie@example.com</t>
+  </si>
+  <si>
+    <t>1122334455</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>david@example.com</t>
+  </si>
+  <si>
+    <t>2233445566</t>
+  </si>
+  <si>
+    <t>Eve</t>
+  </si>
+  <si>
+    <t>eve@example.com</t>
+  </si>
+  <si>
+    <t>3344556677</t>
+  </si>
+  <si>
+    <t>Frank</t>
+  </si>
+  <si>
+    <t>frank@example.com</t>
+  </si>
+  <si>
+    <t>4455667788</t>
+  </si>
+  <si>
+    <t>Grace</t>
+  </si>
+  <si>
+    <t>grace@example.com</t>
+  </si>
+  <si>
+    <t>5566778899</t>
+  </si>
+  <si>
+    <t>Heidi</t>
+  </si>
+  <si>
+    <t>heidi@example.com</t>
+  </si>
+  <si>
+    <t>6677889900</t>
+  </si>
+  <si>
+    <t>Ivan</t>
+  </si>
+  <si>
+    <t>ivan@example.com</t>
+  </si>
+  <si>
+    <t>7788990011</t>
+  </si>
+  <si>
+    <t>Judy</t>
+  </si>
+  <si>
+    <t>judy@example.com</t>
+  </si>
+  <si>
+    <t>8899001122</t>
   </si>
 </sst>
 </file>
@@ -390,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -448,6 +502,72 @@
         <v>14</v>
       </c>
     </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>